<commit_message>
feat: add production profile summary dashboard with EUR calculations and interactive visualizations
</commit_message>
<xml_diff>
--- a/Profile Summary.xlsx
+++ b/Profile Summary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EID1025782\OneDrive - Eni\Documents\PYTHON\ProSum\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EID1025782\OneDrive - Eni\Documents\PYTHON\RESPRO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75989684-2747-407C-B6C5-F16B3143F135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E31A0463-1061-4089-AB78-D8BEA5EA06B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Profile" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId5"/>
+    <pivotCache cacheId="1" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1964" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1973" uniqueCount="60">
   <si>
     <t>Year</t>
   </si>
@@ -219,6 +219,12 @@
   <si>
     <t>Ranggas</t>
   </si>
+  <si>
+    <t>Facility</t>
+  </si>
+  <si>
+    <t>KNH FPSO</t>
+  </si>
 </sst>
 </file>
 
@@ -226,7 +232,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -375,7 +381,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="2" applyBorder="1"/>
@@ -2294,7 +2300,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A5:C19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="6">
     <pivotField axis="axisRow" numFmtId="15" showAll="0">
@@ -15580,10 +15586,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>1</v>
       </c>
@@ -15600,22 +15606,25 @@
         <v>18</v>
       </c>
       <c r="F1" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="G1" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -15628,14 +15637,17 @@
       <c r="E2" s="7">
         <v>46935</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G2">
         <v>9</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>1.778</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -15648,14 +15660,17 @@
       <c r="E3" s="7">
         <v>46935</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G3">
         <v>15</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>4.12</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -15668,14 +15683,17 @@
       <c r="E4" s="7">
         <v>47118</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G4">
         <v>5</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>2.6360000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -15688,14 +15706,17 @@
       <c r="E5" s="7">
         <v>47088</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G5">
         <v>11</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>5.3789999999999996</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -15711,14 +15732,17 @@
       <c r="E6" s="7">
         <v>47118</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G6">
         <v>5</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>2.6360000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -15734,14 +15758,17 @@
       <c r="E7" s="7">
         <v>47088</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G7">
         <v>11</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>5.3789999999999996</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -15757,14 +15784,17 @@
       <c r="E8" s="7">
         <v>47118</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G8">
         <v>5</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>2.6360000000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -15780,10 +15810,13 @@
       <c r="E9" s="7">
         <v>47088</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G9">
         <v>11</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>5.3789999999999996</v>
       </c>
     </row>

</xml_diff>